<commit_message>
fix veille fix pdf
</commit_message>
<xml_diff>
--- a/assets/docs/Synthese_Epreuve_E5_2025.xlsx
+++ b/assets/docs/Synthese_Epreuve_E5_2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ilan.dahan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ilan.dahan/Desktop/iPortfolio/assets/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6850D156-0183-914C-A126-2BB4BC47F773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0430B8D2-2B88-9F4F-8838-AA592888496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="45">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -120,9 +120,6 @@
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>SESSION 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> SLAM</t>
   </si>
   <si>
@@ -178,6 +175,21 @@
   </si>
   <si>
     <t>NOM et prénom : Dahan Ilan</t>
+  </si>
+  <si>
+    <t>Refonte et optumisation du site web de l'entreprise</t>
+  </si>
+  <si>
+    <t>SESSION 2026</t>
+  </si>
+  <si>
+    <t>Creation de base de donnée</t>
+  </si>
+  <si>
+    <t>Devlopement de script pyhton</t>
+  </si>
+  <si>
+    <t>09-2024-05-2025</t>
   </si>
 </sst>
 </file>
@@ -187,7 +199,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -255,6 +267,16 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -655,7 +677,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -720,9 +742,65 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -747,61 +825,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1121,81 +1152,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="H1" s="22"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="31"/>
     </row>
     <row r="2" spans="1:43" ht="41" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="29" t="s">
+      <c r="A3" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="30"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="50"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="A4" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="48"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
       <c r="G4" s="15"/>
       <c r="H4" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="A5" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="38" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1218,8 +1249,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="32"/>
-      <c r="B7" s="40"/>
+      <c r="A7" s="30"/>
+      <c r="B7" s="39"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1275,16 +1306,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.15">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="34"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1323,24 +1354,24 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>30</v>
+      <c r="G9" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="53" t="s">
+        <v>29</v>
       </c>
       <c r="I9"/>
       <c r="J9"/>
@@ -1380,24 +1411,24 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" s="17"/>
-      <c r="D10" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>30</v>
+      <c r="D10" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="53" t="s">
+        <v>29</v>
       </c>
       <c r="I10"/>
       <c r="J10"/>
@@ -1437,22 +1468,22 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="18" t="s">
-        <v>30</v>
+      <c r="E11" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="52"/>
+      <c r="G11" s="52" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="53" t="s">
+        <v>29</v>
       </c>
       <c r="I11"/>
       <c r="J11"/>
@@ -1492,25 +1523,23 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="18" t="s">
-        <v>27</v>
-      </c>
+      <c r="E12" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="53"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1548,25 +1577,27 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="44" t="s">
+      <c r="A13" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="49" t="s">
-        <v>37</v>
-      </c>
       <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F13" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="18" t="s">
-        <v>27</v>
+      <c r="D13" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="53" t="s">
+        <v>26</v>
       </c>
       <c r="I13"/>
       <c r="J13"/>
@@ -1605,14 +1636,26 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
+      <c r="A14" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="18"/>
+      <c r="F14" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="53"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1650,14 +1693,22 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>44</v>
+      </c>
       <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
+      <c r="D15" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
+      <c r="F15" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="G15" s="17"/>
-      <c r="H15" s="18"/>
+      <c r="H15" s="53"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1702,7 +1753,7 @@
       <c r="E16" s="17"/>
       <c r="F16" s="17"/>
       <c r="G16" s="17"/>
-      <c r="H16" s="18"/>
+      <c r="H16" s="53"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1747,7 +1798,7 @@
       <c r="E17" s="17"/>
       <c r="F17" s="17"/>
       <c r="G17" s="17"/>
-      <c r="H17" s="18"/>
+      <c r="H17" s="53"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1792,7 +1843,7 @@
       <c r="E18" s="17"/>
       <c r="F18" s="17"/>
       <c r="G18" s="17"/>
-      <c r="H18" s="18"/>
+      <c r="H18" s="53"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1830,16 +1881,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.15">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="38"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="37"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1877,23 +1928,25 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="44" t="s">
+      <c r="A20" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>26</v>
-      </c>
       <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>27</v>
+      <c r="D20" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="H20" s="53" t="s">
+        <v>26</v>
       </c>
       <c r="I20"/>
       <c r="J20"/>
@@ -2202,16 +2255,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.15">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="48"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="27"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="28"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2249,23 +2302,25 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="45" t="s">
-        <v>28</v>
+      <c r="A28" s="23" t="s">
+        <v>27</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
+      <c r="D28" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="E28" s="17"/>
-      <c r="F28" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G28" s="17" t="s">
-        <v>27</v>
+      <c r="F28" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="52" t="s">
+        <v>26</v>
       </c>
       <c r="H28" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I28"/>
       <c r="J28"/>
@@ -2304,21 +2359,23 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="45" t="s">
-        <v>38</v>
+      <c r="A29" s="23" t="s">
+        <v>37</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C29" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" s="17"/>
+        <v>32</v>
+      </c>
+      <c r="C29" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="52" t="s">
+        <v>26</v>
+      </c>
       <c r="E29" s="17"/>
-      <c r="F29" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G29" s="17"/>
+      <c r="F29" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" s="52"/>
       <c r="H29" s="18"/>
       <c r="I29"/>
       <c r="J29"/>
@@ -2357,22 +2414,24 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="50" t="s">
-        <v>39</v>
+      <c r="A30" s="25" t="s">
+        <v>38</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17" t="s">
-        <v>27</v>
+        <v>32</v>
+      </c>
+      <c r="C30" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="52" t="s">
+        <v>26</v>
       </c>
       <c r="F30" s="17"/>
-      <c r="G30" s="17" t="s">
-        <v>27</v>
+      <c r="G30" s="52" t="s">
+        <v>26</v>
       </c>
       <c r="H30" s="18"/>
       <c r="I30"/>
@@ -2412,11 +2471,17 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="11"/>
+      <c r="A31" s="11" t="s">
+        <v>40</v>
+      </c>
       <c r="B31" s="10"/>
       <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
+      <c r="D31" s="52" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" s="51" t="s">
+        <v>26</v>
+      </c>
       <c r="F31" s="17"/>
       <c r="G31" s="17"/>
       <c r="H31" s="18"/>
@@ -2594,6 +2659,11 @@
     <row r="79" customFormat="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
@@ -2601,11 +2671,6 @@
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>